<commit_message>
#110 #108  Updated Files
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/JLCPCB-BOM-v2.1.xlsx
+++ b/Deliverables/BOM/JLCPCB-BOM-v2.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1D3A9E-6DE5-47E8-84D8-4522C4B46240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7D2585-21E0-4599-BDD8-047D3D4F7976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,24 +16,11 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="133">
   <si>
     <t>Comment</t>
   </si>
@@ -86,6 +73,12 @@
     <t>U262-061N-4BVC11</t>
   </si>
   <si>
+    <t>SPM0687LR5H-1</t>
+  </si>
+  <si>
+    <t>SPH8878LR5H-1</t>
+  </si>
+  <si>
     <t>100K</t>
   </si>
   <si>
@@ -119,9 +112,21 @@
     <t>XC6220B331MR-G</t>
   </si>
   <si>
+    <t>ADS131M08IPBSR</t>
+  </si>
+  <si>
     <t>PCM1865DBTR</t>
   </si>
   <si>
+    <t>UMH3N</t>
+  </si>
+  <si>
+    <t>TLV320ADC5140IRTWT</t>
+  </si>
+  <si>
+    <t>MAX4063ETE+T</t>
+  </si>
+  <si>
     <t>3TJ481920NYLBC</t>
   </si>
   <si>
@@ -188,6 +193,12 @@
     <t>J2</t>
   </si>
   <si>
+    <t>MK1, MK2, MK3, MK4, MK5, MK6, MK7, MK8</t>
+  </si>
+  <si>
+    <t>MK9, MK10, MK11, MK12</t>
+  </si>
+  <si>
     <t>P1</t>
   </si>
   <si>
@@ -224,9 +235,21 @@
     <t>U3</t>
   </si>
   <si>
+    <t>U4</t>
+  </si>
+  <si>
     <t>U5, U6</t>
   </si>
   <si>
+    <t>U13</t>
+  </si>
+  <si>
+    <t>U15</t>
+  </si>
+  <si>
+    <t>U16, U17, U18, U19</t>
+  </si>
+  <si>
     <t>X1</t>
   </si>
   <si>
@@ -278,6 +301,15 @@
     <t>SOT-25</t>
   </si>
   <si>
+    <t>32TQFP</t>
+  </si>
+  <si>
+    <t>24-WQFN (4x4)</t>
+  </si>
+  <si>
+    <t>16-TQFN (4x4)</t>
+  </si>
+  <si>
     <t>LCSC Part Number</t>
   </si>
   <si>
@@ -356,6 +388,9 @@
     <t>C492404</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>C37208</t>
   </si>
   <si>
@@ -375,6 +410,9 @@
   </si>
   <si>
     <t>C181312</t>
+  </si>
+  <si>
+    <t>C123008</t>
   </si>
   <si>
     <t>C2898996</t>
@@ -542,7 +580,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -564,6 +602,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -858,7 +899,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -872,13 +913,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="36" x14ac:dyDescent="0.25">
@@ -886,13 +927,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -900,13 +941,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
@@ -914,13 +955,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -928,13 +969,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -942,13 +983,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -956,13 +997,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -970,13 +1011,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -984,13 +1025,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -998,13 +1039,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1012,13 +1053,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1026,13 +1067,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1040,13 +1081,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1054,13 +1095,13 @@
         <v>6</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1068,13 +1109,13 @@
         <v>9</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1082,13 +1123,13 @@
         <v>9</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -1096,13 +1137,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1110,13 +1151,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -1124,13 +1165,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1138,55 +1179,55 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>91</v>
+      <c r="D20" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+      <c r="A21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="6">
         <v>61300611121</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>92</v>
+      <c r="B23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1194,27 +1235,27 @@
         <v>19</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -1222,13 +1263,13 @@
         <v>21</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="24" x14ac:dyDescent="0.25">
@@ -1236,13 +1277,13 @@
         <v>22</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1250,41 +1291,41 @@
         <v>23</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="24" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>111</v>
+      <c r="B29" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>96</v>
+      <c r="B30" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1292,13 +1333,13 @@
         <v>26</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>79</v>
+        <v>26</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1306,27 +1347,27 @@
         <v>27</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D32" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1334,27 +1375,111 @@
         <v>29</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>115</v>
+      <c r="B35" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>